<commit_message>
Tighten module audit target mappings
</commit_message>
<xml_diff>
--- a/reports/module-data-integration-audit/2026-07-27/CANONICAL_PROMOTION_MATRIX.xlsx
+++ b/reports/module-data-integration-audit/2026-07-27/CANONICAL_PROMOTION_MATRIX.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion" sheetId="1" r:id="R4e5217e0ef5e4237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion" sheetId="1" r:id="Re96849bccc4544fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -310,12 +310,13 @@
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="39" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -326,21 +327,24 @@
         <x:v>schema_table</x:v>
       </x:c>
       <x:c r="C1" s="9" t="str">
-        <x:v>canonical_equivalent</x:v>
+        <x:v>provisional_canonical_object_family</x:v>
       </x:c>
       <x:c r="D1" s="9" t="str">
+        <x:v>mapping_confidence</x:v>
+      </x:c>
+      <x:c r="E1" s="9" t="str">
         <x:v>promotion_trigger</x:v>
       </x:c>
-      <x:c r="E1" s="9" t="str">
+      <x:c r="F1" s="9" t="str">
         <x:v>required_crosswalk</x:v>
       </x:c>
-      <x:c r="F1" s="9" t="str">
+      <x:c r="G1" s="9" t="str">
         <x:v>lineage_required</x:v>
       </x:c>
-      <x:c r="G1" s="9" t="str">
+      <x:c r="H1" s="9" t="str">
         <x:v>complexity</x:v>
       </x:c>
-      <x:c r="H1" s="9" t="str">
+      <x:c r="I1" s="9" t="str">
         <x:v>blocker</x:v>
       </x:c>
     </x:row>
@@ -355,18 +359,21 @@
         <x:v>knowledge.evidence</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E2" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F2" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G2" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H2" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I2" s="5" t="str"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="5" t="str">
@@ -379,18 +386,21 @@
         <x:v>knowledge.evidence</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H3" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H3" s="5" t="str"/>
+      <x:c r="I3" s="5" t="str"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="5" t="str">
@@ -403,18 +413,21 @@
         <x:v>knowledge.evidence_chunk</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="5" t="str">
@@ -427,18 +440,21 @@
         <x:v>knowledge.fact</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H5" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I5" s="5" t="str"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="str">
@@ -448,21 +464,24 @@
         <x:v>public.source_contract_evidence_manifests</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.evidence_manifest</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H6" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H6" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I6" s="5" t="str"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="5" t="str">
@@ -472,21 +491,24 @@
         <x:v>public.source_contract_evidence_metrics</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.metric_observation</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F7" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G7" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I7" s="5" t="str"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="5" t="str">
@@ -496,21 +518,24 @@
         <x:v>public.source_contract_evidence_rows</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.evidence_fragment_or_contract_fact_assertion</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G8" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H8" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H8" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I8" s="5" t="str"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="5" t="str">
@@ -520,21 +545,24 @@
         <x:v>public.source_contract_optimization_findings</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.contract_finding</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G9" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H9" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I9" s="5" t="str"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="5" t="str">
@@ -544,21 +572,24 @@
         <x:v>public.source_contract_optimization_levers</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.value_driver_or_commercial_lever</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H10" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I10" s="5" t="str"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="5" t="str">
@@ -568,21 +599,24 @@
         <x:v>public.source_contract_optimization_profiles</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
-        <x:v>knowledge.contract</x:v>
+        <x:v>knowledge.contract_profile</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H11" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H11" s="5" t="str"/>
+      <x:c r="I11" s="5" t="str"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
@@ -595,18 +629,21 @@
         <x:v>knowledge.fact</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H12" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H12" s="5" t="str"/>
+      <x:c r="I12" s="5" t="str"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
@@ -616,21 +653,24 @@
         <x:v>public.source_meeting_outcomes</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>to_be_mapped_after_live_profile</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>unresolved</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G13" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H13" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H13" s="5" t="str"/>
+      <x:c r="I13" s="5" t="str"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
@@ -640,21 +680,24 @@
         <x:v>public.source_value_chain</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>knowledge.value_flow_step</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E14" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F14" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G14" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H14" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H14" s="5" t="str"/>
+      <x:c r="I14" s="5" t="str"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
@@ -664,21 +707,24 @@
         <x:v>public.source_value_levers</x:v>
       </x:c>
       <x:c r="C15" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>knowledge.value_driver_or_lever</x:v>
       </x:c>
       <x:c r="D15" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G15" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H15" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H15" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I15" s="5" t="str"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
@@ -688,21 +734,24 @@
         <x:v>public.source_value_lines</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>to_be_mapped_after_live_profile</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>unresolved</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G16" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H16" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H16" s="5" t="str"/>
+      <x:c r="I16" s="5" t="str"/>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
@@ -712,21 +761,24 @@
         <x:v>public.source_value_states</x:v>
       </x:c>
       <x:c r="C17" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>knowledge.value_state_or_readiness</x:v>
       </x:c>
       <x:c r="D17" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E17" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F17" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H17" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H17" s="5" t="str"/>
+      <x:c r="I17" s="5" t="str"/>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="5" t="str">
@@ -736,21 +788,24 @@
         <x:v>public.source_vendor_commitments</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
-        <x:v>knowledge.vendor</x:v>
+        <x:v>knowledge.commercial_commitment</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H18" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H18" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I18" s="5" t="str"/>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="5" t="str">
@@ -760,21 +815,24 @@
         <x:v>public.source_vendor_proposal_facts</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
-        <x:v>knowledge.vendor</x:v>
+        <x:v>knowledge.proposal_fact_assertion</x:v>
       </x:c>
       <x:c r="D19" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E19" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F19" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G19" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H19" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H19" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I19" s="5" t="str"/>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="5" t="str">
@@ -784,21 +842,24 @@
         <x:v>public.vendor_contracts</x:v>
       </x:c>
       <x:c r="C20" s="5" t="str">
-        <x:v>knowledge.vendor</x:v>
+        <x:v>knowledge.contract</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E20" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G20" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H20" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H20" s="5" t="str">
+      <x:c r="I20" s="5" t="str">
         <x:v>Lineage field not found statically</x:v>
       </x:c>
     </x:row>
@@ -813,18 +874,21 @@
         <x:v>knowledge.metric_definition</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E21" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G21" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H21" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H21" s="5" t="str"/>
+      <x:c r="I21" s="5" t="str"/>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="5" t="str">
@@ -834,21 +898,24 @@
         <x:v>cio_tower.tool_identity_aliases</x:v>
       </x:c>
       <x:c r="C22" s="5" t="str">
-        <x:v>to_be_mapped</x:v>
+        <x:v>to_be_mapped_after_live_profile</x:v>
       </x:c>
       <x:c r="D22" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>unresolved</x:v>
       </x:c>
       <x:c r="E22" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F22" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G22" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H22" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H22" s="5" t="str"/>
+      <x:c r="I22" s="5" t="str"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="5" t="str">
@@ -858,21 +925,24 @@
         <x:v>public.ai_control_actions</x:v>
       </x:c>
       <x:c r="C23" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.action_or_decision</x:v>
       </x:c>
       <x:c r="D23" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E23" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F23" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G23" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H23" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H23" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I23" s="5" t="str"/>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="5" t="str">
@@ -882,21 +952,24 @@
         <x:v>public.ai_control_agent_outcomes</x:v>
       </x:c>
       <x:c r="C24" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>knowledge.outcome</x:v>
       </x:c>
       <x:c r="D24" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E24" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F24" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G24" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H24" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H24" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I24" s="5" t="str"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="5" t="str">
@@ -906,21 +979,24 @@
         <x:v>public.ai_control_benefit_realization</x:v>
       </x:c>
       <x:c r="C25" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.metric_observation</x:v>
       </x:c>
       <x:c r="D25" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E25" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F25" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G25" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H25" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H25" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I25" s="5" t="str"/>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="5" t="str">
@@ -930,21 +1006,24 @@
         <x:v>public.ai_control_context_facts</x:v>
       </x:c>
       <x:c r="C26" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.fact_assertion</x:v>
       </x:c>
       <x:c r="D26" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E26" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F26" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G26" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H26" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H26" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I26" s="5" t="str"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="5" t="str">
@@ -954,21 +1033,24 @@
         <x:v>public.ai_control_context_relationships</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.relationship_assertion</x:v>
       </x:c>
       <x:c r="D27" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E27" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F27" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G27" s="5" t="str">
-        <x:v>High</x:v>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
       </x:c>
       <x:c r="H27" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I27" s="5" t="str">
         <x:v>Lineage field not found statically</x:v>
       </x:c>
     </x:row>
@@ -980,21 +1062,24 @@
         <x:v>public.ai_control_dora_metrics</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
-        <x:v>knowledge.metric</x:v>
+        <x:v>knowledge.metric_observation</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E28" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F28" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G28" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H28" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H28" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I28" s="5" t="str"/>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="5" t="str">
@@ -1004,21 +1089,24 @@
         <x:v>public.ai_control_evidence_items</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.evidence</x:v>
       </x:c>
       <x:c r="D29" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E29" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F29" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G29" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H29" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H29" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I29" s="5" t="str"/>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="5" t="str">
@@ -1031,18 +1119,21 @@
         <x:v>knowledge.program</x:v>
       </x:c>
       <x:c r="D30" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E30" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F30" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G30" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H30" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H30" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I30" s="5" t="str"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="5" t="str">
@@ -1052,21 +1143,24 @@
         <x:v>public.ai_control_persona_productivity</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.metric_observation</x:v>
       </x:c>
       <x:c r="D31" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E31" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G31" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H31" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H31" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I31" s="5" t="str"/>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="5" t="str">
@@ -1079,18 +1173,21 @@
         <x:v>knowledge.risk_control</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E32" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G32" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H32" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H32" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I32" s="5" t="str"/>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="5" t="str">
@@ -1103,18 +1200,21 @@
         <x:v>knowledge.contract</x:v>
       </x:c>
       <x:c r="D33" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E33" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F33" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G33" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H33" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H33" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I33" s="5" t="str"/>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="5" t="str">
@@ -1124,21 +1224,24 @@
         <x:v>public.ai_control_tool_usage_monthly</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str">
-        <x:v>knowledge.risk_control</x:v>
+        <x:v>knowledge.metric_observation</x:v>
       </x:c>
       <x:c r="D34" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E34" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F34" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G34" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H34" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H34" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I34" s="5" t="str"/>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="5" t="str">
@@ -1151,18 +1254,21 @@
         <x:v>knowledge.application</x:v>
       </x:c>
       <x:c r="D35" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E35" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F35" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G35" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H35" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H35" s="5" t="str">
+      <x:c r="I35" s="5" t="str">
         <x:v>Lineage field not found statically</x:v>
       </x:c>
     </x:row>
@@ -1174,21 +1280,24 @@
         <x:v>public.enterprise_context_records</x:v>
       </x:c>
       <x:c r="C36" s="5" t="str">
-        <x:v>to_be_mapped</x:v>
+        <x:v>to_be_mapped_after_live_profile</x:v>
       </x:c>
       <x:c r="D36" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>unresolved</x:v>
       </x:c>
       <x:c r="E36" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F36" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G36" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H36" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H36" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I36" s="5" t="str"/>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="5" t="str">
@@ -1201,18 +1310,21 @@
         <x:v>knowledge.application</x:v>
       </x:c>
       <x:c r="D37" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E37" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F37" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G37" s="5" t="str">
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H37" s="5" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H37" s="5" t="str"/>
+      <x:c r="I37" s="5" t="str"/>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="5" t="str">
@@ -1225,18 +1337,21 @@
         <x:v>knowledge.vendor</x:v>
       </x:c>
       <x:c r="D38" s="5" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E38" s="5" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F38" s="5" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G38" s="5" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H38" s="5" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H38" s="5" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I38" s="5" t="str"/>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="6" t="str">
@@ -1249,18 +1364,21 @@
         <x:v>knowledge.program</x:v>
       </x:c>
       <x:c r="D39" s="6" t="str">
-        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
+        <x:v>provisional</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
-        <x:v>governance.object_identity_map</x:v>
+        <x:v>Approved/accepted/published state plus evidence lineage and tenant identity verified</x:v>
       </x:c>
       <x:c r="F39" s="6" t="str">
-        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+        <x:v>governance.object_identity_map</x:v>
       </x:c>
       <x:c r="G39" s="6" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="H39" s="6" t="str"/>
+        <x:v>source/evidence/provenance fields or outbox payload evidence</x:v>
+      </x:c>
+      <x:c r="H39" s="6" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="I39" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>